<commit_message>
Updated on 12-20-2023 at 09:53
</commit_message>
<xml_diff>
--- a/output/measles_latex.xlsx
+++ b/output/measles_latex.xlsx
@@ -453,16 +453,16 @@
         <v>0.3101</v>
       </c>
       <c r="C2" t="n">
-        <v>138</v>
+        <v>68</v>
       </c>
       <c r="D2" t="n">
-        <v>2500</v>
+        <v>1639</v>
       </c>
       <c r="E2" t="n">
-        <v>437</v>
+        <v>230</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -473,16 +473,16 @@
         <v>0.2455</v>
       </c>
       <c r="C3" t="n">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="D3" t="n">
-        <v>6563</v>
+        <v>3386</v>
       </c>
       <c r="E3" t="n">
-        <v>1071</v>
+        <v>544</v>
       </c>
       <c r="F3" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -493,13 +493,13 @@
         <v>0.1758</v>
       </c>
       <c r="C4" t="n">
-        <v>162</v>
+        <v>62</v>
       </c>
       <c r="D4" t="n">
-        <v>5287</v>
+        <v>2114</v>
       </c>
       <c r="E4" t="n">
-        <v>1100</v>
+        <v>374</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -513,13 +513,13 @@
         <v>0.09995999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>127</v>
+        <v>43</v>
       </c>
       <c r="D5" t="n">
-        <v>5252</v>
+        <v>2690</v>
       </c>
       <c r="E5" t="n">
-        <v>1218</v>
+        <v>374</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -530,19 +530,19 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>0.01609</v>
+        <v>0.0161</v>
       </c>
       <c r="C6" t="n">
-        <v>465</v>
+        <v>65</v>
       </c>
       <c r="D6" t="n">
-        <v>8929</v>
+        <v>1362</v>
       </c>
       <c r="E6" t="n">
-        <v>2674</v>
+        <v>328</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -553,16 +553,16 @@
         <v>0.009974</v>
       </c>
       <c r="C7" t="n">
-        <v>381</v>
+        <v>53</v>
       </c>
       <c r="D7" t="n">
-        <v>2628</v>
+        <v>2305</v>
       </c>
       <c r="E7" t="n">
-        <v>1058</v>
+        <v>408</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -570,19 +570,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0161</v>
+        <v>0.006375</v>
       </c>
       <c r="C8" t="n">
-        <v>608</v>
+        <v>43</v>
       </c>
       <c r="D8" t="n">
-        <v>3714</v>
+        <v>1472</v>
       </c>
       <c r="E8" t="n">
-        <v>1667</v>
+        <v>282</v>
       </c>
       <c r="F8" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -590,19 +590,19 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>0.004561</v>
+        <v>0.00382</v>
       </c>
       <c r="C9" t="n">
-        <v>491</v>
+        <v>35</v>
       </c>
       <c r="D9" t="n">
-        <v>4025</v>
+        <v>2134</v>
       </c>
       <c r="E9" t="n">
-        <v>1805</v>
+        <v>339</v>
       </c>
       <c r="F9" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -610,19 +610,19 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>0.004982</v>
+        <v>0.003156</v>
       </c>
       <c r="C10" t="n">
-        <v>539</v>
+        <v>64</v>
       </c>
       <c r="D10" t="n">
-        <v>4393</v>
+        <v>1740</v>
       </c>
       <c r="E10" t="n">
-        <v>2135</v>
+        <v>380</v>
       </c>
       <c r="F10" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -630,19 +630,19 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>0.004059</v>
+        <v>0.00264</v>
       </c>
       <c r="C11" t="n">
-        <v>473</v>
+        <v>87</v>
       </c>
       <c r="D11" t="n">
-        <v>9232</v>
+        <v>2527</v>
       </c>
       <c r="E11" t="n">
-        <v>3318</v>
+        <v>365</v>
       </c>
       <c r="F11" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -650,19 +650,19 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>0.003008</v>
+        <v>0.002055</v>
       </c>
       <c r="C12" t="n">
-        <v>557</v>
+        <v>86</v>
       </c>
       <c r="D12" t="n">
-        <v>14186</v>
+        <v>1536</v>
       </c>
       <c r="E12" t="n">
-        <v>4386</v>
+        <v>396</v>
       </c>
       <c r="F12" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>